<commit_message>
fix(frontend): alinhar BACKEND_URL e endurecer proxy; remover fallbacks diretos; ajustar client
</commit_message>
<xml_diff>
--- a/resultado_detran_organizado.xlsx
+++ b/resultado_detran_organizado.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -527,12 +527,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>V608149002</t>
+          <t>A600545200</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -542,12 +542,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>31/01/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>29/05/2026</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -562,12 +562,12 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>DETRAN-CE / CIRETRAN</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -582,27 +582,27 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>N000392817</t>
+          <t>N000429801</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>V607902958</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>MULTA, POR NAO IDENTIFICACAO DO CONDUTOR INFRATOR,</t>
+          <t>N000429801 V608149002 MULTA, POR NAO IDENTIFICACAO DO CONDUTOR INFRATOR,</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>21/01/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>29/05/2026</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -617,12 +617,12 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>DETRAN-CE / CIRETRAN</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -637,12 +637,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>E020019696</t>
+          <t>V608149002</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -652,12 +652,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>20/01/2026</t>
+          <t>31/01/2026</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Órgão cod. 213190</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -692,47 +692,47 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>V020140234</t>
+          <t>N000392817</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>TRANSITAR EM VELOCIDADE SUPERIOR A MAXIMA PERMITID</t>
+          <t>N000392817 V607902958 MULTA, POR NAO IDENTIFICACAO DO CONDUTOR INFRATOR,</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>04/01/2026</t>
+          <t>21/01/2026</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>R$ 130,16</t>
+          <t>R$ 260,32</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>R$ 131,46</t>
+          <t>R$ 262,92</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Órgão cod. 215370</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -747,47 +747,47 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>N000383543</t>
+          <t>E020019696</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>V607859098</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>MULTA, POR NAO IDENTIFICACAO DO CONDUTOR INFRATOR,</t>
+          <t>TRANSITAR EM VELOCIDADE SUPERIOR A MAXIMA PERMITID</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>29/12/2025</t>
+          <t>20/01/2026</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>R$ 260,32</t>
+          <t>R$ 130,16</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>R$ 208,26</t>
+          <t>R$ 131,46</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>DETRAN-CE / CIRETRAN</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -802,47 +802,47 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>N000382394</t>
+          <t>V020140234</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>V607846621</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>MULTA, POR NAO IDENTIFICACAO DO CONDUTOR INFRATOR,</t>
+          <t>TRANSITAR EM VELOCIDADE SUPERIOR A MAXIMA PERMITID</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>29/12/2025</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>R$ 260,32</t>
+          <t>R$ 130,16</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>R$ 208,26</t>
+          <t>R$ 132,88</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>DETRAN-CE / CIRETRAN</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -857,47 +857,47 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>V020129672</t>
+          <t>N000383543</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>TRANSITAR EM VELOCIDADE SUPERIOR A MAXIMA PERMITID</t>
+          <t>N000383543 V607859098 MULTA, POR NAO IDENTIFICACAO DO CONDUTOR INFRATOR,</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>04/12/2025</t>
+          <t>29/12/2025</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>12/02/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>R$ 130,16</t>
+          <t>R$ 260,32</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>R$ 131,46</t>
+          <t>R$ 262,92</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Órgão cod. 215370</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -912,47 +912,47 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>V020126357</t>
+          <t>N000382394</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>TRANSITAR EM VELOCIDADE SUPERIOR A MAXIMA PERMITID</t>
+          <t>N000382394 V607846621 MULTA, POR NAO IDENTIFICACAO DO CONDUTOR INFRATOR,</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>25/11/2025</t>
+          <t>29/12/2025</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>05/02/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>R$ 130,16</t>
+          <t>R$ 260,32</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>R$ 131,46</t>
+          <t>R$ 262,92</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Órgão cod. 215370</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -967,12 +967,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>V607902958</t>
+          <t>V020129672</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -982,12 +982,12 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>02/11/2025</t>
+          <t>04/12/2025</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>12/02/2026</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -997,17 +997,17 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>R$ 131,46</t>
+          <t>R$ 134,46</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>DETRAN-CE / CIRETRAN</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>V020114744</t>
+          <t>V020126357</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1037,12 +1037,12 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>24/10/2025</t>
+          <t>25/11/2025</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>05/02/2026</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -1052,17 +1052,17 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>R$ 132,76</t>
+          <t>R$ 134,46</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Órgão cod. 215370</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -1077,12 +1077,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>V607859098</t>
+          <t>V607902958</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1092,12 +1092,12 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>14/10/2025</t>
+          <t>02/11/2025</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>10/02/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -1107,17 +1107,17 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>R$ 131,46</t>
+          <t>R$ 132,88</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>DETRAN-CE / CIRETRAN</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1132,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>V607846621</t>
+          <t>V020114744</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1147,12 +1147,12 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>24/10/2025</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>09/02/2026</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1162,17 +1162,17 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>R$ 131,46</t>
+          <t>R$ 135,76</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>DETRAN-CE / CIRETRAN</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1187,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>V020107516</t>
+          <t>V607859098</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1202,32 +1202,32 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>14/10/2025</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>18/12/2025</t>
+          <t>10/02/2026</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>R$ 195,23</t>
+          <t>R$ 130,16</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>R$ 201,40</t>
+          <t>R$ 134,46</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Órgão cod. 215370</t>
+          <t>DEMUTRAN RUSSAS</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>
@@ -1242,47 +1242,157 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
+          <t>V607846621</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>TRANSITAR EM VELOCIDADE SUPERIOR A MAXIMA PERMITID</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2025</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>R$ 130,16</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>R$ 134,46</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>DEMUTRAN RUSSAS</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>TIF1J98</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>V020107516</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>TRANSITAR EM VELOCIDADE SUPERIOR A MAXIMA PERMITID</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2025</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>18/12/2025</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>R$ 195,23</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>R$ 205,89</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>DEMUTRAN RUSSAS</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>TIF1J98</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
           <t>V020098768</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>TRANSITAR EM VELOCIDADE SUPERIOR A MAXIMA PERMITID</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>14/09/2025</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>24/11/2025</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>R$ 130,16</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>R$ 135,86</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>Órgão cod. 215370</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>R$ 138,85</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>DEMUTRAN RUSSAS</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>00020101021226850014br.gov.bcb.pix2563pix.santander.com.br/qr/v2/5f1f1b6c-d0b2-4f3c-b3cf-0e6ce263691b52040000530398654072620.845802BR5907SEFAZCE6011FORTALEZACE62070503***63043BAF | 856500000265 208400062021 605292026891 347030791003 | (R$)</t>
         </is>
       </c>
     </row>

</xml_diff>